<commit_message>
Updated the relative paths and fixed the notebook imports
</commit_message>
<xml_diff>
--- a/merged_data/merged_final.xlsx
+++ b/merged_data/merged_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/PEIRU/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e957e68f4fd644b5/Desktop/Education_Wages_Income/merged_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE0A132-82D9-C64F-955E-72884ED9C738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{EDE0A132-82D9-C64F-955E-72884ED9C738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A24E6C5D-0BAE-443F-BABB-6B18A8598EDB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
     <t>university degree</t>
   </si>
   <si>
-    <t>Avg_hourly_value</t>
+    <t>avg_hourly_value</t>
   </si>
 </sst>
 </file>
@@ -437,18 +437,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +474,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -500,7 +500,7 @@
         <v>17.91333333333333</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -526,7 +526,7 @@
         <v>19.66</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -552,7 +552,7 @@
         <v>12.563333333333331</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -578,7 +578,7 @@
         <v>16.133333333333329</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2018</v>
       </c>
@@ -604,7 +604,7 @@
         <v>19.63</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -630,7 +630,7 @@
         <v>22.643333333333331</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2018</v>
       </c>
@@ -656,7 +656,7 @@
         <v>31.3</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2018</v>
       </c>
@@ -682,7 +682,7 @@
         <v>32.016666666666673</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -708,7 +708,7 @@
         <v>10.718666666666669</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2018</v>
       </c>
@@ -734,7 +734,7 @@
         <v>14.46933333333333</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2018</v>
       </c>
@@ -760,7 +760,7 @@
         <v>4.6066666666666656</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2018</v>
       </c>
@@ -786,7 +786,7 @@
         <v>5.8780000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2018</v>
       </c>
@@ -812,7 +812,7 @@
         <v>12.03733333333334</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2018</v>
       </c>
@@ -838,7 +838,7 @@
         <v>13.56999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2018</v>
       </c>
@@ -864,7 +864,7 @@
         <v>20.943333333333332</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2018</v>
       </c>
@@ -890,7 +890,7 @@
         <v>24.48266666666666</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2019</v>
       </c>
@@ -916,7 +916,7 @@
         <v>18.146666666666661</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2019</v>
       </c>
@@ -942,7 +942,7 @@
         <v>20.25333333333333</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2019</v>
       </c>
@@ -968,7 +968,7 @@
         <v>11.87333333333333</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2019</v>
       </c>
@@ -994,7 +994,7 @@
         <v>16.63666666666667</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2019</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>20.49</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2019</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>23.18</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>30.70666666666666</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2019</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>32.74</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2019</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>12.836</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2019</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>14.090666666666669</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2019</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>4.6480000000000006</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2019</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>8.9726666666666688</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2019</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>11.86333333333333</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2019</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>12.151333333333341</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2019</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>21.734666666666659</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2019</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>24.91866666666667</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2020</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>18.77333333333333</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>21.733333333333331</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2020</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>9.129999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2020</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>17.31666666666667</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2020</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>21.23</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2020</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>24.176666666666659</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2020</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>32.796666666666667</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2020</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>33.76</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2020</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>12.04533333333333</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2020</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>13.57066666666667</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2020</v>
       </c>
@@ -1592,7 +1592,7 @@
         <v>4.0533333333333337</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2020</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>5.9253333333333327</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2020</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>11.593333333333341</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2020</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>11.54533333333333</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2020</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>23.39266666666667</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2020</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>24.838666666666679</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>19.366666666666671</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>21.58666666666667</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>11.05</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>17.47333333333334</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2021</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>21.606666666666669</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -1878,7 +1878,7 @@
         <v>24.256666666666661</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2021</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>32.590000000000003</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2021</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>34.416666666666657</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2021</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>13.201333333333331</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2021</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>15.61466666666667</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2021</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>4.3940000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2021</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>5.4893333333333336</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2021</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>11.68466666666666</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2021</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>13.13933333333333</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2021</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>24.454000000000001</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2021</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>26.844666666666679</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2022</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>20.426666666666669</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2022</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>23.013333333333328</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2022</v>
       </c>
@@ -2216,7 +2216,7 @@
         <v>12.52333333333333</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2022</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>18.510000000000002</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2022</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>23.036666666666669</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2022</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>25.856666666666669</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2022</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>34.5</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2022</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>36.169999999999987</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2022</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>14.589333333333331</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2022</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>17.612000000000009</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2022</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>5.5779999999999994</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2022</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>10.050666666666659</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2022</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>13.81733333333333</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2022</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>16.005333333333329</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2022</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>25.998000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2022</v>
       </c>

</xml_diff>